<commit_message>
[MGT-02] Add lead audit sheet and update task board to resolve review feedback
</commit_message>
<xml_diff>
--- a/docs/sprint2/task-board-sprint2.xlsx
+++ b/docs/sprint2/task-board-sprint2.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Беклог задач" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="87">
-  <si>
-    <t>Таблиця розподілу задач Спринта 2 (Task Board) — Фінальна версія</t>
-  </si>
-  <si>
-    <t>Команда: BMIBM-banking | Продукт: «ФінКит» (онлайн-банкінг для фізичних осіб, finkit) | Стан: Підготовка до Demo / здачі</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="87">
+  <si>
+    <t>Таблиця розподілу задач Спринта 2 (Task Board)</t>
+  </si>
+  <si>
+    <t>Команда: BMIBM-banking | Продукт: «ФінКит» (онлайн-банкінг для фізичних осіб, finkit) | Дата планування: 12.10.2026</t>
   </si>
   <si>
     <t>№</t>
@@ -70,6 +70,9 @@
     <t>готово</t>
   </si>
   <si>
+    <t>docs/sprint2/task-board-sprint2.xlsx</t>
+  </si>
+  <si>
     <t>Пономаренко Р. В.</t>
   </si>
   <si>
@@ -79,6 +82,9 @@
     <t>Перехресний розподіл розділів SRS 1.0 (по 2 аудитори на розділ)</t>
   </si>
   <si>
+    <t>task-board-sprint2.xlsx (аркуш 2)</t>
+  </si>
+  <si>
     <t>Городиська А. А.</t>
   </si>
   <si>
@@ -88,6 +94,9 @@
     <t>Узгодження домовленостей, дедлайнів та Definition of Done</t>
   </si>
   <si>
+    <t>task-board-sprint2.xlsx (аркуш 1)</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
@@ -118,7 +127,7 @@
     <t>2.2</t>
   </si>
   <si>
-    <t>Аудит розділів F, GUI, BL та створення аркуша аудиту ТА</t>
+    <t>Аудит розділів F, GUI, BL та 2-га вичитка U, D (аркуш ТА)</t>
   </si>
   <si>
     <t>ТА</t>
@@ -130,7 +139,7 @@
     <t>2.3</t>
   </si>
   <si>
-    <t>Аудит розділів GUI, BL, U, D та створення аркуша аудиту ІТ</t>
+    <t>Аудит розділів GUI, BL, U, D та 2-га вичитка 1–2, P, S (аркуш ІТ)</t>
   </si>
   <si>
     <t>ІТ</t>
@@ -187,6 +196,12 @@
     <t>Оформлення протоколу ретроспективи (Start / Stop / Continue)</t>
   </si>
   <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>в роботі</t>
+  </si>
+  <si>
     <t>docs/sprint2/retro-sprint2.md</t>
   </si>
   <si>
@@ -266,21 +281,6 @@
   </si>
   <si>
     <t>Зручність навігації, тексти помилок, повнота довідки та API</t>
-  </si>
-  <si>
-    <t>заплановано</t>
-  </si>
-  <si>
-    <t>docs/sprint2/task-board-sprint2.xlsx</t>
-  </si>
-  <si>
-    <t>task-board-sprint2.xlsx (аркуш 2)</t>
-  </si>
-  <si>
-    <t>task-board-sprint2.xlsx (аркуш 1)</t>
-  </si>
-  <si>
-    <t>в роботі</t>
   </si>
 </sst>
 </file>
@@ -290,7 +290,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -335,14 +335,24 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="204"/>
     </font>
     <font>
+      <b/>
       <sz val="10"/>
-      <color rgb="FF6C757D"/>
+      <color rgb="FF0F5132"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="204"/>
@@ -356,7 +366,7 @@
       <charset val="204"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -379,12 +389,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD1E7DD"/>
         <bgColor rgb="FFD1E7DD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8F9FA"/>
-        <bgColor rgb="FFF8F9FA"/>
       </patternFill>
     </fill>
     <fill>
@@ -421,7 +425,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -431,40 +435,44 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -767,11 +775,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="54.109375" customWidth="1"/>
+    <col min="2" max="2" width="52" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
@@ -821,414 +829,443 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="13">
         <v>2</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="13">
         <v>2</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="I5" s="8" t="s">
+      <c r="H5" s="7" t="s">
         <v>16</v>
       </c>
+      <c r="I5" s="7" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="17">
+        <v>1</v>
+      </c>
+      <c r="F6" s="17">
+        <v>1</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="17">
+        <v>1</v>
+      </c>
+      <c r="F7" s="17">
+        <v>1</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="7" t="s">
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="13">
+        <v>12</v>
+      </c>
+      <c r="F8" s="13">
+        <v>12</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D9" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="12">
-        <v>1</v>
-      </c>
-      <c r="F6" s="12">
-        <v>1</v>
-      </c>
-      <c r="G6" s="4" t="s">
+      <c r="E9" s="17">
+        <v>4</v>
+      </c>
+      <c r="F9" s="17">
+        <v>4</v>
+      </c>
+      <c r="G9" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="6" t="s">
+      <c r="H9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="I9" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="17">
+        <v>4</v>
+      </c>
+      <c r="F10" s="17">
+        <v>4</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="I10" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="7" t="s">
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="17">
+        <v>4</v>
+      </c>
+      <c r="F11" s="17">
+        <v>4</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="I11" s="15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="17">
+        <v>3.5</v>
+      </c>
+      <c r="F12" s="17">
+        <v>3.5</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="I12" s="15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D13" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="12">
-        <v>1</v>
-      </c>
-      <c r="F7" s="12">
-        <v>1</v>
-      </c>
-      <c r="G7" s="4" t="s">
+      <c r="E13" s="17">
+        <v>2</v>
+      </c>
+      <c r="F13" s="17">
+        <v>2</v>
+      </c>
+      <c r="G13" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="I7" s="6" t="s">
+      <c r="H13" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="I13" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="17">
+        <v>5</v>
+      </c>
+      <c r="F14" s="17">
+        <v>5</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="I14" s="15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" s="17">
+        <v>6</v>
+      </c>
+      <c r="F15" s="17">
+        <v>6</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="I15" s="15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="17">
+        <v>2</v>
+      </c>
+      <c r="F16" s="17">
+        <v>2</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" s="15" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="11">
-        <v>12</v>
-      </c>
-      <c r="F8" s="11">
-        <v>12</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="7" t="s">
+      <c r="I16" s="15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C17" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D17" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="12">
-        <v>4</v>
-      </c>
-      <c r="F9" s="12">
-        <v>4</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="12">
-        <v>4</v>
-      </c>
-      <c r="F10" s="12">
-        <v>4</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="12">
-        <v>4</v>
-      </c>
-      <c r="F11" s="12">
-        <v>4</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I11" s="6" t="s">
+      <c r="E17" s="17">
+        <v>1.5</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="15" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E12" s="12">
-        <v>3.5</v>
-      </c>
-      <c r="F12" s="12">
-        <v>3.5</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="12">
-        <v>2</v>
-      </c>
-      <c r="F13" s="12">
-        <v>2</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E14" s="12">
-        <v>5</v>
-      </c>
-      <c r="F14" s="12">
-        <v>5</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="12">
-        <v>6</v>
-      </c>
-      <c r="F15" s="12">
-        <v>6</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E16" s="12">
-        <v>2</v>
-      </c>
-      <c r="F16" s="12">
-        <v>2</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E17" s="12">
+      <c r="E18" s="17">
         <v>1.5</v>
       </c>
-      <c r="F17" s="12">
-        <v>1.5</v>
-      </c>
-      <c r="G17" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E18" s="12">
-        <v>1.5</v>
-      </c>
-      <c r="F18" s="12">
-        <v>1.5</v>
-      </c>
-      <c r="G18" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="H18" s="6" t="s">
+      <c r="F18" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="I18" s="6" t="s">
-        <v>16</v>
+      <c r="G18" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="H18" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="I18" s="15" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" s="18"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" s="18"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1249,131 +1286,131 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>69</v>
+      <c r="A5" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>74</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D6" s="7" t="s">
+      <c r="A6" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>73</v>
       </c>
+      <c r="D6" s="6" t="s">
+        <v>78</v>
+      </c>
       <c r="E6" s="4" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="E7" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="7" t="s">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="6" t="s">
+      <c r="D9" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>73</v>
-      </c>
       <c r="E10" s="4" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>